<commit_message>
26/04/2026: Due to errors in data, which is used in modeling, an extensive review was made to ensure that output data will be valid for use, and it’s as follows: -	Change backward fill to be forward fill in all functions to avoid filling with false data which will have bad impact on the later steps -	Remove section 2.4. -	Enhance yahoo finance function to deal with first two days in 2016 which weren’t trading days. -	Change place for gold volatility index to be after FRED function. -	Added first finished trials of AI modeling.
</commit_message>
<xml_diff>
--- a/raw data/egy_cbe_inflation_rate.xlsx
+++ b/raw data/egy_cbe_inflation_rate.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="617" uniqueCount="617">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="622" uniqueCount="622">
   <si>
     <t/>
   </si>
@@ -30,6 +30,21 @@
   </si>
   <si>
     <t>Fruits and Vegetables (y/y)</t>
+  </si>
+  <si>
+    <t>Mar 2026</t>
+  </si>
+  <si>
+    <t>15.200%</t>
+  </si>
+  <si>
+    <t>14.000%</t>
+  </si>
+  <si>
+    <t>19.000%</t>
+  </si>
+  <si>
+    <t>15.900%</t>
   </si>
   <si>
     <t>Feb 2026</t>
@@ -1932,7 +1947,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="xr">
-  <dimension ref="A1:E136"/>
+  <dimension ref="A1:E137"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1" style="1"/>
@@ -2024,41 +2039,41 @@
         <v>21</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>22</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>31</v>
@@ -2143,24 +2158,24 @@
         <v>54</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>60</v>
@@ -2350,24 +2365,24 @@
         <v>114</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>86</v>
+        <v>115</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>119</v>
+        <v>91</v>
       </c>
       <c r="D26" s="4" t="s">
         <v>120</v>
@@ -2517,24 +2532,24 @@
         <v>162</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>123</v>
+        <v>163</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>167</v>
+        <v>128</v>
       </c>
       <c r="C36" s="4" t="s">
         <v>168</v>
@@ -3764,24 +3779,24 @@
         <v>528</v>
       </c>
       <c r="D108" s="4" t="s">
-        <v>524</v>
+        <v>529</v>
       </c>
       <c r="E108" s="4" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="4" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="B109" s="4" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="C109" s="4" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="D109" s="4" t="s">
-        <v>533</v>
+        <v>529</v>
       </c>
       <c r="E109" s="4" t="s">
         <v>534</v>
@@ -3798,24 +3813,24 @@
         <v>537</v>
       </c>
       <c r="D110" s="4" t="s">
-        <v>533</v>
+        <v>538</v>
       </c>
       <c r="E110" s="4" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="4" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="B111" s="4" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="C111" s="4" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="D111" s="4" t="s">
-        <v>542</v>
+        <v>538</v>
       </c>
       <c r="E111" s="4" t="s">
         <v>543</v>
@@ -3894,24 +3909,24 @@
         <v>564</v>
       </c>
       <c r="B116" s="4" t="s">
-        <v>407</v>
+        <v>565</v>
       </c>
       <c r="C116" s="4" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="D116" s="4" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="E116" s="4" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="4" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="B117" s="4" t="s">
-        <v>569</v>
+        <v>412</v>
       </c>
       <c r="C117" s="4" t="s">
         <v>570</v>
@@ -3968,24 +3983,24 @@
         <v>585</v>
       </c>
       <c r="D120" s="4" t="s">
-        <v>581</v>
+        <v>586</v>
       </c>
       <c r="E120" s="4" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="4" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="B121" s="4" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="C121" s="4" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="D121" s="4" t="s">
-        <v>590</v>
+        <v>586</v>
       </c>
       <c r="E121" s="4" t="s">
         <v>591</v>
@@ -4042,60 +4057,76 @@
         <v>606</v>
       </c>
     </row>
-    <row r="127">
-      <c r="A127" s="1" t="s">
+    <row r="125">
+      <c r="A125" s="4" t="s">
         <v>607</v>
+      </c>
+      <c r="B125" s="4" t="s">
+        <v>608</v>
+      </c>
+      <c r="C125" s="4" t="s">
+        <v>609</v>
+      </c>
+      <c r="D125" s="4" t="s">
+        <v>610</v>
+      </c>
+      <c r="E125" s="4" t="s">
+        <v>611</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="1" t="s">
-        <v>608</v>
+        <v>612</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="1" t="s">
-        <v>609</v>
+        <v>613</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="1" t="s">
-        <v>610</v>
+        <v>614</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="1" t="s">
-        <v>611</v>
+        <v>615</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="1" t="s">
-        <v>612</v>
+        <v>616</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="1" t="s">
-        <v>613</v>
+        <v>617</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="1" t="s">
-        <v>614</v>
+        <v>618</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="1" t="s">
-        <v>615</v>
+        <v>619</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="1" t="s">
-        <v>616</v>
+        <v>620</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="1" t="s">
+        <v>621</v>
       </c>
     </row>
   </sheetData>
   <mergeCells>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A127:E127"/>
     <mergeCell ref="A128:E128"/>
     <mergeCell ref="A129:E129"/>
     <mergeCell ref="A130:E130"/>
@@ -4105,10 +4136,11 @@
     <mergeCell ref="A134:E134"/>
     <mergeCell ref="A135:E135"/>
     <mergeCell ref="A136:E136"/>
+    <mergeCell ref="A137:E137"/>
   </mergeCells>
   <headerFooter/>
   <ignoredErrors>
-    <ignoredError sqref="A1:E124" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:E125" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>